<commit_message>
feat: 100 yeni kart gorseli — set 100'den 200'e
- 6 Ekim partisi: gorsel-sahneleri.json, ayni recete (seed, stil referansi)
- sete girmeyi sinif degil gorsel belirliyor (32 kurtarilabilir kart girdi)
- kanca panosu tasinca yazdigi sayi cizdigiyle ayni (panoKancalari)
- sitenin vitrin 20 kelimesi acik liste: adresler kaymasin
- recete: %65 ozne, ayak alti golge, 'yalnizca stili kopyala' dersleri

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kart-inceleme.xlsx
+++ b/kart-inceleme.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3542" uniqueCount="1237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3576" uniqueCount="1237">
   <si>
     <t>Sıra</t>
   </si>
@@ -8604,7 +8604,7 @@
         <v>454</v>
       </c>
       <c r="F102" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G102" t="s">
         <v>18</v>
@@ -8624,8 +8624,8 @@
       <c r="L102" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M102">
-        <v>28</v>
+      <c r="M102" t="s">
+        <v>23</v>
       </c>
       <c r="N102" t="s">
         <v>23</v>
@@ -8648,7 +8648,7 @@
         <v>457</v>
       </c>
       <c r="F103" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G103" t="s">
         <v>18</v>
@@ -8668,8 +8668,8 @@
       <c r="L103" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M103">
-        <v>29</v>
+      <c r="M103" t="s">
+        <v>23</v>
       </c>
       <c r="N103" t="s">
         <v>23</v>
@@ -8692,7 +8692,7 @@
         <v>461</v>
       </c>
       <c r="F104" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G104" t="s">
         <v>18</v>
@@ -8712,8 +8712,8 @@
       <c r="L104" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M104">
-        <v>30</v>
+      <c r="M104" t="s">
+        <v>23</v>
       </c>
       <c r="N104" t="s">
         <v>23</v>
@@ -8736,7 +8736,7 @@
         <v>465</v>
       </c>
       <c r="F105" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G105" t="s">
         <v>18</v>
@@ -8756,8 +8756,8 @@
       <c r="L105" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M105">
-        <v>31</v>
+      <c r="M105" t="s">
+        <v>23</v>
       </c>
       <c r="N105" t="s">
         <v>23</v>
@@ -8780,7 +8780,7 @@
         <v>469</v>
       </c>
       <c r="F106" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G106" t="s">
         <v>18</v>
@@ -8800,8 +8800,8 @@
       <c r="L106" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M106">
-        <v>32</v>
+      <c r="M106" t="s">
+        <v>23</v>
       </c>
       <c r="N106" t="s">
         <v>23</v>
@@ -8824,7 +8824,7 @@
         <v>473</v>
       </c>
       <c r="F107" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G107" t="s">
         <v>18</v>
@@ -8844,8 +8844,8 @@
       <c r="L107" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M107">
-        <v>33</v>
+      <c r="M107" t="s">
+        <v>23</v>
       </c>
       <c r="N107" t="s">
         <v>23</v>
@@ -8868,7 +8868,7 @@
         <v>477</v>
       </c>
       <c r="F108" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G108" t="s">
         <v>18</v>
@@ -8888,8 +8888,8 @@
       <c r="L108" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M108">
-        <v>34</v>
+      <c r="M108" t="s">
+        <v>23</v>
       </c>
       <c r="N108" t="s">
         <v>23</v>
@@ -8912,7 +8912,7 @@
         <v>481</v>
       </c>
       <c r="F109" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G109" t="s">
         <v>18</v>
@@ -8932,8 +8932,8 @@
       <c r="L109" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M109">
-        <v>35</v>
+      <c r="M109" t="s">
+        <v>23</v>
       </c>
       <c r="N109" t="s">
         <v>23</v>
@@ -8956,7 +8956,7 @@
         <v>485</v>
       </c>
       <c r="F110" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G110" t="s">
         <v>18</v>
@@ -8976,8 +8976,8 @@
       <c r="L110" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M110">
-        <v>36</v>
+      <c r="M110" t="s">
+        <v>23</v>
       </c>
       <c r="N110" t="s">
         <v>23</v>
@@ -9000,7 +9000,7 @@
         <v>489</v>
       </c>
       <c r="F111" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G111" t="s">
         <v>18</v>
@@ -9020,8 +9020,8 @@
       <c r="L111" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M111">
-        <v>37</v>
+      <c r="M111" t="s">
+        <v>23</v>
       </c>
       <c r="N111" t="s">
         <v>23</v>
@@ -9044,7 +9044,7 @@
         <v>493</v>
       </c>
       <c r="F112" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G112" t="s">
         <v>18</v>
@@ -9064,8 +9064,8 @@
       <c r="L112" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M112">
-        <v>38</v>
+      <c r="M112" t="s">
+        <v>23</v>
       </c>
       <c r="N112" t="s">
         <v>23</v>
@@ -9088,7 +9088,7 @@
         <v>497</v>
       </c>
       <c r="F113" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G113" t="s">
         <v>18</v>
@@ -9108,8 +9108,8 @@
       <c r="L113" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M113">
-        <v>39</v>
+      <c r="M113" t="s">
+        <v>23</v>
       </c>
       <c r="N113" t="s">
         <v>23</v>
@@ -9132,7 +9132,7 @@
         <v>501</v>
       </c>
       <c r="F114" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G114" t="s">
         <v>18</v>
@@ -9152,8 +9152,8 @@
       <c r="L114" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M114">
-        <v>40</v>
+      <c r="M114" t="s">
+        <v>23</v>
       </c>
       <c r="N114" t="s">
         <v>23</v>
@@ -9176,7 +9176,7 @@
         <v>505</v>
       </c>
       <c r="F115" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G115" t="s">
         <v>18</v>
@@ -9196,8 +9196,8 @@
       <c r="L115" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M115">
-        <v>41</v>
+      <c r="M115" t="s">
+        <v>23</v>
       </c>
       <c r="N115" t="s">
         <v>23</v>
@@ -9240,8 +9240,8 @@
       <c r="L116" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M116" t="s">
-        <v>23</v>
+      <c r="M116">
+        <v>27</v>
       </c>
       <c r="N116" t="s">
         <v>23</v>
@@ -9308,7 +9308,7 @@
         <v>518</v>
       </c>
       <c r="F118" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G118" t="s">
         <v>18</v>
@@ -9328,8 +9328,8 @@
       <c r="L118" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M118">
-        <v>42</v>
+      <c r="M118" t="s">
+        <v>23</v>
       </c>
       <c r="N118" t="s">
         <v>23</v>
@@ -9396,7 +9396,7 @@
         <v>527</v>
       </c>
       <c r="F120" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G120" t="s">
         <v>18</v>
@@ -9416,8 +9416,8 @@
       <c r="L120" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M120">
-        <v>43</v>
+      <c r="M120" t="s">
+        <v>23</v>
       </c>
       <c r="N120" t="s">
         <v>23</v>
@@ -9440,7 +9440,7 @@
         <v>531</v>
       </c>
       <c r="F121" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G121" t="s">
         <v>18</v>
@@ -9460,8 +9460,8 @@
       <c r="L121" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M121">
-        <v>44</v>
+      <c r="M121" t="s">
+        <v>23</v>
       </c>
       <c r="N121" t="s">
         <v>23</v>
@@ -9484,7 +9484,7 @@
         <v>535</v>
       </c>
       <c r="F122" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G122" t="s">
         <v>18</v>
@@ -9504,8 +9504,8 @@
       <c r="L122" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M122">
-        <v>1</v>
+      <c r="M122" t="s">
+        <v>23</v>
       </c>
       <c r="N122" t="s">
         <v>23</v>
@@ -9528,7 +9528,7 @@
         <v>540</v>
       </c>
       <c r="F123" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G123" t="s">
         <v>18</v>
@@ -9548,8 +9548,8 @@
       <c r="L123" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M123">
-        <v>45</v>
+      <c r="M123" t="s">
+        <v>23</v>
       </c>
       <c r="N123" t="s">
         <v>23</v>
@@ -9592,8 +9592,8 @@
       <c r="L124" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M124" t="s">
-        <v>23</v>
+      <c r="M124">
+        <v>28</v>
       </c>
       <c r="N124" t="s">
         <v>23</v>
@@ -9616,7 +9616,7 @@
         <v>548</v>
       </c>
       <c r="F125" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G125" t="s">
         <v>18</v>
@@ -9636,8 +9636,8 @@
       <c r="L125" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M125">
-        <v>2</v>
+      <c r="M125" t="s">
+        <v>23</v>
       </c>
       <c r="N125" t="s">
         <v>23</v>
@@ -9660,7 +9660,7 @@
         <v>552</v>
       </c>
       <c r="F126" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G126" t="s">
         <v>18</v>
@@ -9680,8 +9680,8 @@
       <c r="L126" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M126">
-        <v>46</v>
+      <c r="M126" t="s">
+        <v>23</v>
       </c>
       <c r="N126" t="s">
         <v>23</v>
@@ -9724,8 +9724,8 @@
       <c r="L127" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M127" t="s">
-        <v>23</v>
+      <c r="M127">
+        <v>29</v>
       </c>
       <c r="N127" t="s">
         <v>23</v>
@@ -9748,7 +9748,7 @@
         <v>560</v>
       </c>
       <c r="F128" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G128" t="s">
         <v>18</v>
@@ -9768,8 +9768,8 @@
       <c r="L128" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M128">
-        <v>3</v>
+      <c r="M128" t="s">
+        <v>23</v>
       </c>
       <c r="N128" t="s">
         <v>23</v>
@@ -9792,7 +9792,7 @@
         <v>564</v>
       </c>
       <c r="F129" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G129" t="s">
         <v>18</v>
@@ -9812,8 +9812,8 @@
       <c r="L129" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M129">
-        <v>47</v>
+      <c r="M129" t="s">
+        <v>23</v>
       </c>
       <c r="N129" t="s">
         <v>23</v>
@@ -9900,8 +9900,8 @@
       <c r="L131" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M131" t="s">
-        <v>23</v>
+      <c r="M131">
+        <v>30</v>
       </c>
       <c r="N131" t="s">
         <v>23</v>
@@ -9924,7 +9924,7 @@
         <v>577</v>
       </c>
       <c r="F132" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G132" t="s">
         <v>18</v>
@@ -9944,8 +9944,8 @@
       <c r="L132" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M132">
-        <v>4</v>
+      <c r="M132" t="s">
+        <v>23</v>
       </c>
       <c r="N132" t="s">
         <v>23</v>
@@ -9988,8 +9988,8 @@
       <c r="L133" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M133" t="s">
-        <v>23</v>
+      <c r="M133">
+        <v>31</v>
       </c>
       <c r="N133" t="s">
         <v>23</v>
@@ -10012,7 +10012,7 @@
         <v>585</v>
       </c>
       <c r="F134" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G134" t="s">
         <v>18</v>
@@ -10032,8 +10032,8 @@
       <c r="L134" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M134">
-        <v>5</v>
+      <c r="M134" t="s">
+        <v>23</v>
       </c>
       <c r="N134" t="s">
         <v>23</v>
@@ -10056,7 +10056,7 @@
         <v>589</v>
       </c>
       <c r="F135" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G135" t="s">
         <v>18</v>
@@ -10076,8 +10076,8 @@
       <c r="L135" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M135">
-        <v>48</v>
+      <c r="M135" t="s">
+        <v>23</v>
       </c>
       <c r="N135" t="s">
         <v>23</v>
@@ -10144,7 +10144,7 @@
         <v>599</v>
       </c>
       <c r="F137" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G137" t="s">
         <v>18</v>
@@ -10164,8 +10164,8 @@
       <c r="L137" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M137">
-        <v>49</v>
+      <c r="M137" t="s">
+        <v>23</v>
       </c>
       <c r="N137" t="s">
         <v>23</v>
@@ -10208,8 +10208,8 @@
       <c r="L138" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M138" t="s">
-        <v>23</v>
+      <c r="M138">
+        <v>32</v>
       </c>
       <c r="N138" t="s">
         <v>23</v>
@@ -10252,8 +10252,8 @@
       <c r="L139" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M139" t="s">
-        <v>23</v>
+      <c r="M139">
+        <v>33</v>
       </c>
       <c r="N139" t="s">
         <v>23</v>
@@ -10296,8 +10296,8 @@
       <c r="L140" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M140" t="s">
-        <v>23</v>
+      <c r="M140">
+        <v>34</v>
       </c>
       <c r="N140" t="s">
         <v>23</v>
@@ -10320,7 +10320,7 @@
         <v>615</v>
       </c>
       <c r="F141" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G141" t="s">
         <v>92</v>
@@ -10340,8 +10340,8 @@
       <c r="L141" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M141">
-        <v>79</v>
+      <c r="M141" t="s">
+        <v>23</v>
       </c>
       <c r="N141" t="s">
         <v>23</v>
@@ -10364,7 +10364,7 @@
         <v>619</v>
       </c>
       <c r="F142" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G142" t="s">
         <v>18</v>
@@ -10384,8 +10384,8 @@
       <c r="L142" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M142">
-        <v>50</v>
+      <c r="M142" t="s">
+        <v>23</v>
       </c>
       <c r="N142" t="s">
         <v>23</v>
@@ -10408,7 +10408,7 @@
         <v>621</v>
       </c>
       <c r="F143" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G143" t="s">
         <v>18</v>
@@ -10428,8 +10428,8 @@
       <c r="L143" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M143">
-        <v>51</v>
+      <c r="M143" t="s">
+        <v>23</v>
       </c>
       <c r="N143" t="s">
         <v>23</v>
@@ -10472,8 +10472,8 @@
       <c r="L144" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M144" t="s">
-        <v>23</v>
+      <c r="M144">
+        <v>35</v>
       </c>
       <c r="N144" t="s">
         <v>23</v>
@@ -10496,7 +10496,7 @@
         <v>629</v>
       </c>
       <c r="F145" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G145" t="s">
         <v>18</v>
@@ -10516,8 +10516,8 @@
       <c r="L145" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M145">
-        <v>52</v>
+      <c r="M145" t="s">
+        <v>23</v>
       </c>
       <c r="N145" t="s">
         <v>23</v>
@@ -10540,7 +10540,7 @@
         <v>633</v>
       </c>
       <c r="F146" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G146" t="s">
         <v>92</v>
@@ -10560,8 +10560,8 @@
       <c r="L146" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M146">
-        <v>80</v>
+      <c r="M146" t="s">
+        <v>23</v>
       </c>
       <c r="N146" t="s">
         <v>23</v>
@@ -10604,8 +10604,8 @@
       <c r="L147" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M147" t="s">
-        <v>23</v>
+      <c r="M147">
+        <v>36</v>
       </c>
       <c r="N147" t="s">
         <v>23</v>
@@ -10692,8 +10692,8 @@
       <c r="L149" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M149" t="s">
-        <v>23</v>
+      <c r="M149">
+        <v>37</v>
       </c>
       <c r="N149" t="s">
         <v>23</v>
@@ -10716,7 +10716,7 @@
         <v>650</v>
       </c>
       <c r="F150" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G150" t="s">
         <v>92</v>
@@ -10736,8 +10736,8 @@
       <c r="L150" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M150">
-        <v>81</v>
+      <c r="M150" t="s">
+        <v>23</v>
       </c>
       <c r="N150" t="s">
         <v>23</v>
@@ -10760,7 +10760,7 @@
         <v>654</v>
       </c>
       <c r="F151" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G151" t="s">
         <v>18</v>
@@ -10780,8 +10780,8 @@
       <c r="L151" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M151">
-        <v>6</v>
+      <c r="M151" t="s">
+        <v>23</v>
       </c>
       <c r="N151" t="s">
         <v>23</v>
@@ -10804,7 +10804,7 @@
         <v>657</v>
       </c>
       <c r="F152" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G152" t="s">
         <v>92</v>
@@ -10824,8 +10824,8 @@
       <c r="L152" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M152">
-        <v>82</v>
+      <c r="M152" t="s">
+        <v>23</v>
       </c>
       <c r="N152" t="s">
         <v>23</v>
@@ -10848,7 +10848,7 @@
         <v>660</v>
       </c>
       <c r="F153" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G153" t="s">
         <v>92</v>
@@ -10868,8 +10868,8 @@
       <c r="L153" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M153">
-        <v>83</v>
+      <c r="M153" t="s">
+        <v>23</v>
       </c>
       <c r="N153" t="s">
         <v>23</v>
@@ -10980,7 +10980,7 @@
         <v>674</v>
       </c>
       <c r="F156" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G156" t="s">
         <v>18</v>
@@ -11000,8 +11000,8 @@
       <c r="L156" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M156">
-        <v>53</v>
+      <c r="M156" t="s">
+        <v>23</v>
       </c>
       <c r="N156" t="s">
         <v>23</v>
@@ -11044,8 +11044,8 @@
       <c r="L157" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M157" t="s">
-        <v>23</v>
+      <c r="M157">
+        <v>38</v>
       </c>
       <c r="N157" t="s">
         <v>23</v>
@@ -11068,7 +11068,7 @@
         <v>681</v>
       </c>
       <c r="F158" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G158" t="s">
         <v>18</v>
@@ -11088,8 +11088,8 @@
       <c r="L158" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M158">
-        <v>7</v>
+      <c r="M158" t="s">
+        <v>23</v>
       </c>
       <c r="N158" t="s">
         <v>23</v>
@@ -11156,7 +11156,7 @@
         <v>688</v>
       </c>
       <c r="F160" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G160" t="s">
         <v>18</v>
@@ -11176,8 +11176,8 @@
       <c r="L160" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M160">
-        <v>54</v>
+      <c r="M160" t="s">
+        <v>23</v>
       </c>
       <c r="N160" t="s">
         <v>23</v>
@@ -11200,7 +11200,7 @@
         <v>692</v>
       </c>
       <c r="F161" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G161" t="s">
         <v>18</v>
@@ -11220,8 +11220,8 @@
       <c r="L161" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M161">
-        <v>8</v>
+      <c r="M161" t="s">
+        <v>23</v>
       </c>
       <c r="N161" t="s">
         <v>23</v>
@@ -11264,8 +11264,8 @@
       <c r="L162" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M162" t="s">
-        <v>23</v>
+      <c r="M162">
+        <v>39</v>
       </c>
       <c r="N162" t="s">
         <v>23</v>
@@ -11376,7 +11376,7 @@
         <v>709</v>
       </c>
       <c r="F165" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G165" t="s">
         <v>92</v>
@@ -11396,8 +11396,8 @@
       <c r="L165" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M165">
-        <v>84</v>
+      <c r="M165" t="s">
+        <v>23</v>
       </c>
       <c r="N165" t="s">
         <v>23</v>
@@ -11420,7 +11420,7 @@
         <v>712</v>
       </c>
       <c r="F166" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G166" t="s">
         <v>18</v>
@@ -11440,8 +11440,8 @@
       <c r="L166" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M166">
-        <v>9</v>
+      <c r="M166" t="s">
+        <v>23</v>
       </c>
       <c r="N166" t="s">
         <v>23</v>
@@ -11464,7 +11464,7 @@
         <v>716</v>
       </c>
       <c r="F167" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G167" t="s">
         <v>18</v>
@@ -11484,8 +11484,8 @@
       <c r="L167" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M167">
-        <v>55</v>
+      <c r="M167" t="s">
+        <v>23</v>
       </c>
       <c r="N167" t="s">
         <v>23</v>
@@ -11508,7 +11508,7 @@
         <v>720</v>
       </c>
       <c r="F168" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G168" t="s">
         <v>18</v>
@@ -11528,8 +11528,8 @@
       <c r="L168" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M168">
-        <v>56</v>
+      <c r="M168" t="s">
+        <v>23</v>
       </c>
       <c r="N168" t="s">
         <v>23</v>
@@ -11552,7 +11552,7 @@
         <v>724</v>
       </c>
       <c r="F169" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G169" t="s">
         <v>92</v>
@@ -11572,8 +11572,8 @@
       <c r="L169" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M169">
-        <v>85</v>
+      <c r="M169" t="s">
+        <v>23</v>
       </c>
       <c r="N169" t="s">
         <v>23</v>
@@ -11596,7 +11596,7 @@
         <v>728</v>
       </c>
       <c r="F170" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G170" t="s">
         <v>18</v>
@@ -11616,8 +11616,8 @@
       <c r="L170" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M170">
-        <v>10</v>
+      <c r="M170" t="s">
+        <v>23</v>
       </c>
       <c r="N170" t="s">
         <v>23</v>
@@ -11704,8 +11704,8 @@
       <c r="L172" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M172" t="s">
-        <v>23</v>
+      <c r="M172">
+        <v>40</v>
       </c>
       <c r="N172" t="s">
         <v>23</v>
@@ -11728,7 +11728,7 @@
         <v>740</v>
       </c>
       <c r="F173" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G173" t="s">
         <v>18</v>
@@ -11748,8 +11748,8 @@
       <c r="L173" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M173">
-        <v>11</v>
+      <c r="M173" t="s">
+        <v>23</v>
       </c>
       <c r="N173" t="s">
         <v>23</v>
@@ -11792,8 +11792,8 @@
       <c r="L174" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M174" t="s">
-        <v>23</v>
+      <c r="M174">
+        <v>41</v>
       </c>
       <c r="N174" t="s">
         <v>23</v>
@@ -11860,7 +11860,7 @@
         <v>753</v>
       </c>
       <c r="F176" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G176" t="s">
         <v>18</v>
@@ -11880,8 +11880,8 @@
       <c r="L176" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M176">
-        <v>57</v>
+      <c r="M176" t="s">
+        <v>23</v>
       </c>
       <c r="N176" t="s">
         <v>23</v>
@@ -11904,7 +11904,7 @@
         <v>757</v>
       </c>
       <c r="F177" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G177" t="s">
         <v>18</v>
@@ -11924,8 +11924,8 @@
       <c r="L177" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M177">
-        <v>58</v>
+      <c r="M177" t="s">
+        <v>23</v>
       </c>
       <c r="N177" t="s">
         <v>23</v>
@@ -11992,7 +11992,7 @@
         <v>766</v>
       </c>
       <c r="F179" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G179" t="s">
         <v>18</v>
@@ -12012,8 +12012,8 @@
       <c r="L179" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M179">
-        <v>12</v>
+      <c r="M179" t="s">
+        <v>23</v>
       </c>
       <c r="N179" t="s">
         <v>23</v>
@@ -12080,7 +12080,7 @@
         <v>774</v>
       </c>
       <c r="F181" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G181" t="s">
         <v>18</v>
@@ -12100,8 +12100,8 @@
       <c r="L181" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M181">
-        <v>13</v>
+      <c r="M181" t="s">
+        <v>23</v>
       </c>
       <c r="N181" t="s">
         <v>23</v>
@@ -12124,7 +12124,7 @@
         <v>778</v>
       </c>
       <c r="F182" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G182" t="s">
         <v>18</v>
@@ -12144,8 +12144,8 @@
       <c r="L182" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M182">
-        <v>14</v>
+      <c r="M182" t="s">
+        <v>23</v>
       </c>
       <c r="N182" t="s">
         <v>23</v>
@@ -12168,7 +12168,7 @@
         <v>782</v>
       </c>
       <c r="F183" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G183" t="s">
         <v>18</v>
@@ -12188,8 +12188,8 @@
       <c r="L183" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M183">
-        <v>15</v>
+      <c r="M183" t="s">
+        <v>23</v>
       </c>
       <c r="N183" t="s">
         <v>23</v>
@@ -12212,7 +12212,7 @@
         <v>786</v>
       </c>
       <c r="F184" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G184" t="s">
         <v>18</v>
@@ -12232,8 +12232,8 @@
       <c r="L184" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M184">
-        <v>16</v>
+      <c r="M184" t="s">
+        <v>23</v>
       </c>
       <c r="N184" t="s">
         <v>23</v>
@@ -12276,8 +12276,8 @@
       <c r="L185" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M185" t="s">
-        <v>23</v>
+      <c r="M185">
+        <v>42</v>
       </c>
       <c r="N185" t="s">
         <v>23</v>
@@ -12300,7 +12300,7 @@
         <v>794</v>
       </c>
       <c r="F186" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G186" t="s">
         <v>18</v>
@@ -12320,8 +12320,8 @@
       <c r="L186" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M186">
-        <v>17</v>
+      <c r="M186" t="s">
+        <v>23</v>
       </c>
       <c r="N186" t="s">
         <v>23</v>
@@ -12344,7 +12344,7 @@
         <v>797</v>
       </c>
       <c r="F187" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G187" t="s">
         <v>92</v>
@@ -12364,8 +12364,8 @@
       <c r="L187" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M187">
-        <v>86</v>
+      <c r="M187" t="s">
+        <v>23</v>
       </c>
       <c r="N187" t="s">
         <v>23</v>
@@ -12408,8 +12408,8 @@
       <c r="L188" s="3" t="s">
         <v>802</v>
       </c>
-      <c r="M188" t="s">
-        <v>23</v>
+      <c r="M188">
+        <v>43</v>
       </c>
       <c r="N188" t="s">
         <v>23</v>
@@ -12476,7 +12476,7 @@
         <v>810</v>
       </c>
       <c r="F190" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G190" t="s">
         <v>92</v>
@@ -12496,8 +12496,8 @@
       <c r="L190" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M190">
-        <v>87</v>
+      <c r="M190" t="s">
+        <v>23</v>
       </c>
       <c r="N190" t="s">
         <v>23</v>
@@ -12520,7 +12520,7 @@
         <v>814</v>
       </c>
       <c r="F191" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G191" t="s">
         <v>18</v>
@@ -12540,8 +12540,8 @@
       <c r="L191" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M191">
-        <v>59</v>
+      <c r="M191" t="s">
+        <v>23</v>
       </c>
       <c r="N191" t="s">
         <v>23</v>
@@ -12584,8 +12584,8 @@
       <c r="L192" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M192" t="s">
-        <v>23</v>
+      <c r="M192">
+        <v>44</v>
       </c>
       <c r="N192" t="s">
         <v>23</v>
@@ -12608,7 +12608,7 @@
         <v>820</v>
       </c>
       <c r="F193" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G193" t="s">
         <v>92</v>
@@ -12628,8 +12628,8 @@
       <c r="L193" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M193">
-        <v>88</v>
+      <c r="M193" t="s">
+        <v>23</v>
       </c>
       <c r="N193" t="s">
         <v>23</v>
@@ -12652,7 +12652,7 @@
         <v>824</v>
       </c>
       <c r="F194" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G194" t="s">
         <v>92</v>
@@ -12672,8 +12672,8 @@
       <c r="L194" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M194">
-        <v>89</v>
+      <c r="M194" t="s">
+        <v>23</v>
       </c>
       <c r="N194" t="s">
         <v>23</v>
@@ -12760,8 +12760,8 @@
       <c r="L196" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M196" t="s">
-        <v>23</v>
+      <c r="M196">
+        <v>45</v>
       </c>
       <c r="N196" t="s">
         <v>23</v>
@@ -12804,8 +12804,8 @@
       <c r="L197" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M197" t="s">
-        <v>23</v>
+      <c r="M197">
+        <v>46</v>
       </c>
       <c r="N197" t="s">
         <v>23</v>
@@ -12848,8 +12848,8 @@
       <c r="L198" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M198" t="s">
-        <v>23</v>
+      <c r="M198">
+        <v>47</v>
       </c>
       <c r="N198" t="s">
         <v>23</v>
@@ -12872,7 +12872,7 @@
         <v>844</v>
       </c>
       <c r="F199" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G199" t="s">
         <v>18</v>
@@ -12892,8 +12892,8 @@
       <c r="L199" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M199">
-        <v>60</v>
+      <c r="M199" t="s">
+        <v>23</v>
       </c>
       <c r="N199" t="s">
         <v>23</v>
@@ -12936,8 +12936,8 @@
       <c r="L200" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M200" t="s">
-        <v>23</v>
+      <c r="M200">
+        <v>48</v>
       </c>
       <c r="N200" t="s">
         <v>23</v>
@@ -13068,8 +13068,8 @@
       <c r="L203" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M203" t="s">
-        <v>23</v>
+      <c r="M203">
+        <v>49</v>
       </c>
       <c r="N203" t="s">
         <v>23</v>
@@ -13156,8 +13156,8 @@
       <c r="L205" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M205" t="s">
-        <v>23</v>
+      <c r="M205">
+        <v>50</v>
       </c>
       <c r="N205" t="s">
         <v>23</v>
@@ -13180,7 +13180,7 @@
         <v>872</v>
       </c>
       <c r="F206" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G206" t="s">
         <v>92</v>
@@ -13200,8 +13200,8 @@
       <c r="L206" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M206">
-        <v>90</v>
+      <c r="M206" t="s">
+        <v>23</v>
       </c>
       <c r="N206" t="s">
         <v>23</v>
@@ -13244,8 +13244,8 @@
       <c r="L207" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M207" t="s">
-        <v>23</v>
+      <c r="M207">
+        <v>51</v>
       </c>
       <c r="N207" t="s">
         <v>23</v>
@@ -13268,7 +13268,7 @@
         <v>880</v>
       </c>
       <c r="F208" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G208" t="s">
         <v>92</v>
@@ -13288,8 +13288,8 @@
       <c r="L208" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M208">
-        <v>91</v>
+      <c r="M208" t="s">
+        <v>23</v>
       </c>
       <c r="N208" t="s">
         <v>23</v>
@@ -13312,7 +13312,7 @@
         <v>883</v>
       </c>
       <c r="F209" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G209" t="s">
         <v>18</v>
@@ -13332,8 +13332,8 @@
       <c r="L209" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M209">
-        <v>18</v>
+      <c r="M209" t="s">
+        <v>23</v>
       </c>
       <c r="N209" t="s">
         <v>23</v>
@@ -13356,7 +13356,7 @@
         <v>887</v>
       </c>
       <c r="F210" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G210" t="s">
         <v>18</v>
@@ -13376,8 +13376,8 @@
       <c r="L210" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M210">
-        <v>19</v>
+      <c r="M210" t="s">
+        <v>23</v>
       </c>
       <c r="N210" t="s">
         <v>23</v>
@@ -13400,7 +13400,7 @@
         <v>890</v>
       </c>
       <c r="F211" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G211" t="s">
         <v>18</v>
@@ -13420,8 +13420,8 @@
       <c r="L211" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M211">
-        <v>20</v>
+      <c r="M211" t="s">
+        <v>23</v>
       </c>
       <c r="N211" t="s">
         <v>23</v>
@@ -13488,7 +13488,7 @@
         <v>899</v>
       </c>
       <c r="F213" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G213" t="s">
         <v>18</v>
@@ -13508,8 +13508,8 @@
       <c r="L213" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M213">
-        <v>61</v>
+      <c r="M213" t="s">
+        <v>23</v>
       </c>
       <c r="N213" t="s">
         <v>23</v>
@@ -13552,8 +13552,8 @@
       <c r="L214" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M214" t="s">
-        <v>23</v>
+      <c r="M214">
+        <v>52</v>
       </c>
       <c r="N214" t="s">
         <v>23</v>
@@ -13576,7 +13576,7 @@
         <v>907</v>
       </c>
       <c r="F215" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G215" t="s">
         <v>92</v>
@@ -13596,8 +13596,8 @@
       <c r="L215" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M215">
-        <v>92</v>
+      <c r="M215" t="s">
+        <v>23</v>
       </c>
       <c r="N215" t="s">
         <v>23</v>
@@ -13620,7 +13620,7 @@
         <v>911</v>
       </c>
       <c r="F216" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G216" t="s">
         <v>92</v>
@@ -13640,8 +13640,8 @@
       <c r="L216" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M216">
-        <v>93</v>
+      <c r="M216" t="s">
+        <v>23</v>
       </c>
       <c r="N216" t="s">
         <v>23</v>
@@ -13684,8 +13684,8 @@
       <c r="L217" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M217" t="s">
-        <v>23</v>
+      <c r="M217">
+        <v>53</v>
       </c>
       <c r="N217" t="s">
         <v>23</v>
@@ -13708,7 +13708,7 @@
         <v>919</v>
       </c>
       <c r="F218" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G218" t="s">
         <v>18</v>
@@ -13728,8 +13728,8 @@
       <c r="L218" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M218">
-        <v>62</v>
+      <c r="M218" t="s">
+        <v>23</v>
       </c>
       <c r="N218" t="s">
         <v>23</v>
@@ -13752,7 +13752,7 @@
         <v>921</v>
       </c>
       <c r="F219" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G219" t="s">
         <v>92</v>
@@ -13772,8 +13772,8 @@
       <c r="L219" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M219">
-        <v>94</v>
+      <c r="M219" t="s">
+        <v>23</v>
       </c>
       <c r="N219" t="s">
         <v>23</v>
@@ -13840,7 +13840,7 @@
         <v>930</v>
       </c>
       <c r="F221" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G221" t="s">
         <v>18</v>
@@ -13860,8 +13860,8 @@
       <c r="L221" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M221">
-        <v>63</v>
+      <c r="M221" t="s">
+        <v>23</v>
       </c>
       <c r="N221" t="s">
         <v>23</v>
@@ -13884,7 +13884,7 @@
         <v>934</v>
       </c>
       <c r="F222" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G222" t="s">
         <v>18</v>
@@ -13904,8 +13904,8 @@
       <c r="L222" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M222">
-        <v>64</v>
+      <c r="M222" t="s">
+        <v>23</v>
       </c>
       <c r="N222" t="s">
         <v>23</v>
@@ -13928,7 +13928,7 @@
         <v>938</v>
       </c>
       <c r="F223" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G223" t="s">
         <v>92</v>
@@ -13948,8 +13948,8 @@
       <c r="L223" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M223">
-        <v>95</v>
+      <c r="M223" t="s">
+        <v>23</v>
       </c>
       <c r="N223" t="s">
         <v>23</v>
@@ -13972,7 +13972,7 @@
         <v>942</v>
       </c>
       <c r="F224" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G224" t="s">
         <v>18</v>
@@ -13992,8 +13992,8 @@
       <c r="L224" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M224">
-        <v>65</v>
+      <c r="M224" t="s">
+        <v>23</v>
       </c>
       <c r="N224" t="s">
         <v>23</v>
@@ -14016,7 +14016,7 @@
         <v>944</v>
       </c>
       <c r="F225" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G225" t="s">
         <v>92</v>
@@ -14036,8 +14036,8 @@
       <c r="L225" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M225">
-        <v>96</v>
+      <c r="M225" t="s">
+        <v>23</v>
       </c>
       <c r="N225" t="s">
         <v>23</v>
@@ -14060,7 +14060,7 @@
         <v>948</v>
       </c>
       <c r="F226" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G226" t="s">
         <v>92</v>
@@ -14080,8 +14080,8 @@
       <c r="L226" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M226">
-        <v>97</v>
+      <c r="M226" t="s">
+        <v>23</v>
       </c>
       <c r="N226" t="s">
         <v>23</v>
@@ -14104,7 +14104,7 @@
         <v>951</v>
       </c>
       <c r="F227" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G227" t="s">
         <v>92</v>
@@ -14124,8 +14124,8 @@
       <c r="L227" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M227">
-        <v>98</v>
+      <c r="M227" t="s">
+        <v>23</v>
       </c>
       <c r="N227" t="s">
         <v>23</v>
@@ -14148,7 +14148,7 @@
         <v>954</v>
       </c>
       <c r="F228" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G228" t="s">
         <v>92</v>
@@ -14168,8 +14168,8 @@
       <c r="L228" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M228">
-        <v>99</v>
+      <c r="M228" t="s">
+        <v>23</v>
       </c>
       <c r="N228" t="s">
         <v>23</v>
@@ -14280,7 +14280,7 @@
         <v>967</v>
       </c>
       <c r="F231" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G231" t="s">
         <v>18</v>
@@ -14300,8 +14300,8 @@
       <c r="L231" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M231">
-        <v>66</v>
+      <c r="M231" t="s">
+        <v>23</v>
       </c>
       <c r="N231" t="s">
         <v>23</v>
@@ -14344,8 +14344,8 @@
       <c r="L232" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M232" t="s">
-        <v>23</v>
+      <c r="M232">
+        <v>54</v>
       </c>
       <c r="N232" t="s">
         <v>23</v>
@@ -14368,7 +14368,7 @@
         <v>974</v>
       </c>
       <c r="F233" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G233" t="s">
         <v>92</v>
@@ -14388,8 +14388,8 @@
       <c r="L233" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M233">
-        <v>100</v>
+      <c r="M233" t="s">
+        <v>23</v>
       </c>
       <c r="N233" t="s">
         <v>23</v>
@@ -14432,8 +14432,8 @@
       <c r="L234" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M234" t="s">
-        <v>23</v>
+      <c r="M234">
+        <v>1</v>
       </c>
       <c r="N234" t="s">
         <v>23</v>
@@ -14456,7 +14456,7 @@
         <v>981</v>
       </c>
       <c r="F235" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G235" t="s">
         <v>18</v>
@@ -14476,8 +14476,8 @@
       <c r="L235" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M235">
-        <v>67</v>
+      <c r="M235" t="s">
+        <v>23</v>
       </c>
       <c r="N235" t="s">
         <v>23</v>
@@ -14544,7 +14544,7 @@
         <v>990</v>
       </c>
       <c r="F237" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G237" t="s">
         <v>18</v>
@@ -14564,8 +14564,8 @@
       <c r="L237" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M237">
-        <v>68</v>
+      <c r="M237" t="s">
+        <v>23</v>
       </c>
       <c r="N237" t="s">
         <v>23</v>
@@ -14588,7 +14588,7 @@
         <v>994</v>
       </c>
       <c r="F238" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G238" t="s">
         <v>18</v>
@@ -14608,8 +14608,8 @@
       <c r="L238" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M238">
-        <v>21</v>
+      <c r="M238" t="s">
+        <v>23</v>
       </c>
       <c r="N238" t="s">
         <v>23</v>
@@ -14652,8 +14652,8 @@
       <c r="L239" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M239" t="s">
-        <v>23</v>
+      <c r="M239">
+        <v>2</v>
       </c>
       <c r="N239" t="s">
         <v>23</v>
@@ -14696,8 +14696,8 @@
       <c r="L240" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M240" t="s">
-        <v>23</v>
+      <c r="M240">
+        <v>3</v>
       </c>
       <c r="N240" t="s">
         <v>23</v>
@@ -14740,8 +14740,8 @@
       <c r="L241" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M241" t="s">
-        <v>23</v>
+      <c r="M241">
+        <v>4</v>
       </c>
       <c r="N241" t="s">
         <v>23</v>
@@ -14872,8 +14872,8 @@
       <c r="L244" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M244" t="s">
-        <v>23</v>
+      <c r="M244">
+        <v>55</v>
       </c>
       <c r="N244" t="s">
         <v>23</v>
@@ -15004,8 +15004,8 @@
       <c r="L247" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M247" t="s">
-        <v>23</v>
+      <c r="M247">
+        <v>5</v>
       </c>
       <c r="N247" t="s">
         <v>23</v>
@@ -15048,8 +15048,8 @@
       <c r="L248" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M248" t="s">
-        <v>23</v>
+      <c r="M248">
+        <v>6</v>
       </c>
       <c r="N248" t="s">
         <v>23</v>
@@ -15180,8 +15180,8 @@
       <c r="L251" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M251" t="s">
-        <v>23</v>
+      <c r="M251">
+        <v>7</v>
       </c>
       <c r="N251" t="s">
         <v>23</v>
@@ -15204,7 +15204,7 @@
         <v>1049</v>
       </c>
       <c r="F252" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G252" t="s">
         <v>18</v>
@@ -15224,8 +15224,8 @@
       <c r="L252" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M252">
-        <v>22</v>
+      <c r="M252" t="s">
+        <v>23</v>
       </c>
       <c r="N252" t="s">
         <v>23</v>
@@ -15268,8 +15268,8 @@
       <c r="L253" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M253" t="s">
-        <v>23</v>
+      <c r="M253">
+        <v>56</v>
       </c>
       <c r="N253" t="s">
         <v>23</v>
@@ -15312,8 +15312,8 @@
       <c r="L254" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M254" t="s">
-        <v>23</v>
+      <c r="M254">
+        <v>8</v>
       </c>
       <c r="N254" t="s">
         <v>23</v>
@@ -15400,8 +15400,8 @@
       <c r="L256" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M256" t="s">
-        <v>23</v>
+      <c r="M256">
+        <v>57</v>
       </c>
       <c r="N256" t="s">
         <v>23</v>
@@ -15444,8 +15444,8 @@
       <c r="L257" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M257" t="s">
-        <v>23</v>
+      <c r="M257">
+        <v>9</v>
       </c>
       <c r="N257" t="s">
         <v>23</v>
@@ -15488,8 +15488,8 @@
       <c r="L258" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M258" t="s">
-        <v>23</v>
+      <c r="M258">
+        <v>10</v>
       </c>
       <c r="N258" t="s">
         <v>23</v>
@@ -15532,8 +15532,8 @@
       <c r="L259" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M259" t="s">
-        <v>23</v>
+      <c r="M259">
+        <v>11</v>
       </c>
       <c r="N259" t="s">
         <v>23</v>
@@ -15576,8 +15576,8 @@
       <c r="L260" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M260" t="s">
-        <v>23</v>
+      <c r="M260">
+        <v>58</v>
       </c>
       <c r="N260" t="s">
         <v>23</v>
@@ -15620,8 +15620,8 @@
       <c r="L261" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M261" t="s">
-        <v>23</v>
+      <c r="M261">
+        <v>12</v>
       </c>
       <c r="N261" t="s">
         <v>23</v>
@@ -15664,8 +15664,8 @@
       <c r="L262" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M262" t="s">
-        <v>23</v>
+      <c r="M262">
+        <v>13</v>
       </c>
       <c r="N262" t="s">
         <v>23</v>
@@ -15688,7 +15688,7 @@
         <v>1088</v>
       </c>
       <c r="F263" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G263" t="s">
         <v>18</v>
@@ -15708,8 +15708,8 @@
       <c r="L263" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M263">
-        <v>69</v>
+      <c r="M263" t="s">
+        <v>23</v>
       </c>
       <c r="N263" t="s">
         <v>23</v>
@@ -15752,8 +15752,8 @@
       <c r="L264" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M264" t="s">
-        <v>23</v>
+      <c r="M264">
+        <v>59</v>
       </c>
       <c r="N264" t="s">
         <v>23</v>
@@ -15796,8 +15796,8 @@
       <c r="L265" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M265" t="s">
-        <v>23</v>
+      <c r="M265">
+        <v>60</v>
       </c>
       <c r="N265" t="s">
         <v>23</v>
@@ -15820,7 +15820,7 @@
         <v>1098</v>
       </c>
       <c r="F266" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G266" t="s">
         <v>18</v>
@@ -15840,7 +15840,7 @@
       <c r="L266" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M266">
+      <c r="M266" t="s">
         <v>23</v>
       </c>
       <c r="N266" t="s">
@@ -15884,8 +15884,8 @@
       <c r="L267" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M267" t="s">
-        <v>23</v>
+      <c r="M267">
+        <v>14</v>
       </c>
       <c r="N267" t="s">
         <v>23</v>
@@ -15928,8 +15928,8 @@
       <c r="L268" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M268" t="s">
-        <v>23</v>
+      <c r="M268">
+        <v>15</v>
       </c>
       <c r="N268" t="s">
         <v>23</v>
@@ -15952,7 +15952,7 @@
         <v>1109</v>
       </c>
       <c r="F269" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G269" t="s">
         <v>18</v>
@@ -15972,8 +15972,8 @@
       <c r="L269" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M269">
-        <v>24</v>
+      <c r="M269" t="s">
+        <v>23</v>
       </c>
       <c r="N269" t="s">
         <v>23</v>
@@ -16016,8 +16016,8 @@
       <c r="L270" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M270" t="s">
-        <v>23</v>
+      <c r="M270">
+        <v>16</v>
       </c>
       <c r="N270" t="s">
         <v>23</v>
@@ -16040,7 +16040,7 @@
         <v>1116</v>
       </c>
       <c r="F271" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G271" t="s">
         <v>18</v>
@@ -16060,8 +16060,8 @@
       <c r="L271" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M271">
-        <v>70</v>
+      <c r="M271" t="s">
+        <v>23</v>
       </c>
       <c r="N271" t="s">
         <v>23</v>
@@ -16084,7 +16084,7 @@
         <v>1120</v>
       </c>
       <c r="F272" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G272" t="s">
         <v>18</v>
@@ -16104,8 +16104,8 @@
       <c r="L272" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M272">
-        <v>71</v>
+      <c r="M272" t="s">
+        <v>23</v>
       </c>
       <c r="N272" t="s">
         <v>23</v>
@@ -16128,7 +16128,7 @@
         <v>1124</v>
       </c>
       <c r="F273" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G273" t="s">
         <v>18</v>
@@ -16148,8 +16148,8 @@
       <c r="L273" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M273">
-        <v>72</v>
+      <c r="M273" t="s">
+        <v>23</v>
       </c>
       <c r="N273" t="s">
         <v>23</v>
@@ -16172,7 +16172,7 @@
         <v>1128</v>
       </c>
       <c r="F274" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G274" t="s">
         <v>18</v>
@@ -16192,8 +16192,8 @@
       <c r="L274" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M274">
-        <v>73</v>
+      <c r="M274" t="s">
+        <v>23</v>
       </c>
       <c r="N274" t="s">
         <v>23</v>
@@ -16216,7 +16216,7 @@
         <v>1132</v>
       </c>
       <c r="F275" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G275" t="s">
         <v>18</v>
@@ -16236,8 +16236,8 @@
       <c r="L275" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M275">
-        <v>74</v>
+      <c r="M275" t="s">
+        <v>23</v>
       </c>
       <c r="N275" t="s">
         <v>23</v>
@@ -16260,7 +16260,7 @@
         <v>1136</v>
       </c>
       <c r="F276" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G276" t="s">
         <v>18</v>
@@ -16280,8 +16280,8 @@
       <c r="L276" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M276">
-        <v>75</v>
+      <c r="M276" t="s">
+        <v>23</v>
       </c>
       <c r="N276" t="s">
         <v>23</v>
@@ -16324,8 +16324,8 @@
       <c r="L277" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M277" t="s">
-        <v>23</v>
+      <c r="M277">
+        <v>17</v>
       </c>
       <c r="N277" t="s">
         <v>23</v>
@@ -16368,8 +16368,8 @@
       <c r="L278" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M278" t="s">
-        <v>23</v>
+      <c r="M278">
+        <v>18</v>
       </c>
       <c r="N278" t="s">
         <v>23</v>
@@ -16412,8 +16412,8 @@
       <c r="L279" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M279" t="s">
-        <v>23</v>
+      <c r="M279">
+        <v>61</v>
       </c>
       <c r="N279" t="s">
         <v>23</v>
@@ -16500,8 +16500,8 @@
       <c r="L281" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M281" t="s">
-        <v>23</v>
+      <c r="M281">
+        <v>62</v>
       </c>
       <c r="N281" t="s">
         <v>23</v>
@@ -16524,7 +16524,7 @@
         <v>1158</v>
       </c>
       <c r="F282" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G282" t="s">
         <v>18</v>
@@ -16544,8 +16544,8 @@
       <c r="L282" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M282">
-        <v>25</v>
+      <c r="M282" t="s">
+        <v>23</v>
       </c>
       <c r="N282" t="s">
         <v>23</v>
@@ -16588,8 +16588,8 @@
       <c r="L283" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M283" t="s">
-        <v>23</v>
+      <c r="M283">
+        <v>63</v>
       </c>
       <c r="N283" t="s">
         <v>23</v>
@@ -16612,7 +16612,7 @@
         <v>1166</v>
       </c>
       <c r="F284" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G284" t="s">
         <v>18</v>
@@ -16632,8 +16632,8 @@
       <c r="L284" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M284">
-        <v>26</v>
+      <c r="M284" t="s">
+        <v>23</v>
       </c>
       <c r="N284" t="s">
         <v>23</v>
@@ -16676,8 +16676,8 @@
       <c r="L285" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M285" t="s">
-        <v>23</v>
+      <c r="M285">
+        <v>19</v>
       </c>
       <c r="N285" t="s">
         <v>23</v>
@@ -16700,7 +16700,7 @@
         <v>1172</v>
       </c>
       <c r="F286" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G286" t="s">
         <v>18</v>
@@ -16720,8 +16720,8 @@
       <c r="L286" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M286">
-        <v>76</v>
+      <c r="M286" t="s">
+        <v>23</v>
       </c>
       <c r="N286" t="s">
         <v>23</v>
@@ -16744,7 +16744,7 @@
         <v>1175</v>
       </c>
       <c r="F287" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G287" t="s">
         <v>18</v>
@@ -16764,8 +16764,8 @@
       <c r="L287" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M287">
-        <v>27</v>
+      <c r="M287" t="s">
+        <v>23</v>
       </c>
       <c r="N287" t="s">
         <v>23</v>
@@ -16788,7 +16788,7 @@
         <v>1179</v>
       </c>
       <c r="F288" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G288" t="s">
         <v>18</v>
@@ -16808,8 +16808,8 @@
       <c r="L288" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M288">
-        <v>77</v>
+      <c r="M288" t="s">
+        <v>23</v>
       </c>
       <c r="N288" t="s">
         <v>23</v>
@@ -16832,7 +16832,7 @@
         <v>1183</v>
       </c>
       <c r="F289" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G289" t="s">
         <v>18</v>
@@ -16852,8 +16852,8 @@
       <c r="L289" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M289">
-        <v>78</v>
+      <c r="M289" t="s">
+        <v>23</v>
       </c>
       <c r="N289" t="s">
         <v>23</v>
@@ -16896,8 +16896,8 @@
       <c r="L290" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M290" t="s">
-        <v>23</v>
+      <c r="M290">
+        <v>20</v>
       </c>
       <c r="N290" t="s">
         <v>23</v>
@@ -16940,8 +16940,8 @@
       <c r="L291" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M291" t="s">
-        <v>23</v>
+      <c r="M291">
+        <v>21</v>
       </c>
       <c r="N291" t="s">
         <v>23</v>
@@ -16984,8 +16984,8 @@
       <c r="L292" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M292" t="s">
-        <v>23</v>
+      <c r="M292">
+        <v>22</v>
       </c>
       <c r="N292" t="s">
         <v>23</v>
@@ -17072,7 +17072,7 @@
       <c r="L294" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M294" t="s">
+      <c r="M294">
         <v>23</v>
       </c>
       <c r="N294" t="s">
@@ -17116,8 +17116,8 @@
       <c r="L295" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M295" t="s">
-        <v>23</v>
+      <c r="M295">
+        <v>24</v>
       </c>
       <c r="N295" t="s">
         <v>23</v>
@@ -17204,8 +17204,8 @@
       <c r="L297" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M297" t="s">
-        <v>23</v>
+      <c r="M297">
+        <v>64</v>
       </c>
       <c r="N297" t="s">
         <v>23</v>
@@ -17248,8 +17248,8 @@
       <c r="L298" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M298" t="s">
-        <v>23</v>
+      <c r="M298">
+        <v>65</v>
       </c>
       <c r="N298" t="s">
         <v>23</v>
@@ -17292,8 +17292,8 @@
       <c r="L299" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M299" t="s">
-        <v>23</v>
+      <c r="M299">
+        <v>25</v>
       </c>
       <c r="N299" t="s">
         <v>23</v>
@@ -17336,8 +17336,8 @@
       <c r="L300" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M300" t="s">
-        <v>23</v>
+      <c r="M300">
+        <v>26</v>
       </c>
       <c r="N300" t="s">
         <v>23</v>
@@ -17380,8 +17380,8 @@
       <c r="L301" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M301" t="s">
-        <v>23</v>
+      <c r="M301">
+        <v>66</v>
       </c>
       <c r="N301" t="s">
         <v>23</v>
@@ -17415,7 +17415,7 @@
         <v>1231</v>
       </c>
       <c r="B2">
-        <v>100</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -17479,7 +17479,7 @@
         <v>1236</v>
       </c>
       <c r="B13">
-        <v>166</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat: 66 kart gorseli daha — set 200'den 266'ya
Uretime hazir kartlarin tamami (tanidik/odunc kelimeler agirlikli).
Kalan 34 kart duzeltme bekliyor ya da kalite 1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kart-inceleme.xlsx
+++ b/kart-inceleme.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3576" uniqueCount="1237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3642" uniqueCount="1237">
   <si>
     <t>Sıra</t>
   </si>
@@ -9220,7 +9220,7 @@
         <v>509</v>
       </c>
       <c r="F116" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G116" t="s">
         <v>92</v>
@@ -9240,8 +9240,8 @@
       <c r="L116" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M116">
-        <v>27</v>
+      <c r="M116" t="s">
+        <v>23</v>
       </c>
       <c r="N116" t="s">
         <v>23</v>
@@ -9572,7 +9572,7 @@
         <v>544</v>
       </c>
       <c r="F124" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G124" t="s">
         <v>92</v>
@@ -9592,8 +9592,8 @@
       <c r="L124" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M124">
-        <v>28</v>
+      <c r="M124" t="s">
+        <v>23</v>
       </c>
       <c r="N124" t="s">
         <v>23</v>
@@ -9704,7 +9704,7 @@
         <v>556</v>
       </c>
       <c r="F127" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G127" t="s">
         <v>92</v>
@@ -9724,8 +9724,8 @@
       <c r="L127" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M127">
-        <v>29</v>
+      <c r="M127" t="s">
+        <v>23</v>
       </c>
       <c r="N127" t="s">
         <v>23</v>
@@ -9880,7 +9880,7 @@
         <v>573</v>
       </c>
       <c r="F131" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G131" t="s">
         <v>92</v>
@@ -9900,8 +9900,8 @@
       <c r="L131" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M131">
-        <v>30</v>
+      <c r="M131" t="s">
+        <v>23</v>
       </c>
       <c r="N131" t="s">
         <v>23</v>
@@ -9968,7 +9968,7 @@
         <v>581</v>
       </c>
       <c r="F133" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G133" t="s">
         <v>92</v>
@@ -9988,8 +9988,8 @@
       <c r="L133" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M133">
-        <v>31</v>
+      <c r="M133" t="s">
+        <v>23</v>
       </c>
       <c r="N133" t="s">
         <v>23</v>
@@ -10188,7 +10188,7 @@
         <v>603</v>
       </c>
       <c r="F138" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G138" t="s">
         <v>92</v>
@@ -10208,8 +10208,8 @@
       <c r="L138" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M138">
-        <v>32</v>
+      <c r="M138" t="s">
+        <v>23</v>
       </c>
       <c r="N138" t="s">
         <v>23</v>
@@ -10232,7 +10232,7 @@
         <v>607</v>
       </c>
       <c r="F139" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G139" t="s">
         <v>92</v>
@@ -10252,8 +10252,8 @@
       <c r="L139" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M139">
-        <v>33</v>
+      <c r="M139" t="s">
+        <v>23</v>
       </c>
       <c r="N139" t="s">
         <v>23</v>
@@ -10276,7 +10276,7 @@
         <v>611</v>
       </c>
       <c r="F140" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G140" t="s">
         <v>92</v>
@@ -10296,8 +10296,8 @@
       <c r="L140" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M140">
-        <v>34</v>
+      <c r="M140" t="s">
+        <v>23</v>
       </c>
       <c r="N140" t="s">
         <v>23</v>
@@ -10452,7 +10452,7 @@
         <v>625</v>
       </c>
       <c r="F144" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G144" t="s">
         <v>92</v>
@@ -10472,8 +10472,8 @@
       <c r="L144" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M144">
-        <v>35</v>
+      <c r="M144" t="s">
+        <v>23</v>
       </c>
       <c r="N144" t="s">
         <v>23</v>
@@ -10584,7 +10584,7 @@
         <v>637</v>
       </c>
       <c r="F147" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G147" t="s">
         <v>92</v>
@@ -10604,8 +10604,8 @@
       <c r="L147" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M147">
-        <v>36</v>
+      <c r="M147" t="s">
+        <v>23</v>
       </c>
       <c r="N147" t="s">
         <v>23</v>
@@ -10672,7 +10672,7 @@
         <v>646</v>
       </c>
       <c r="F149" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G149" t="s">
         <v>92</v>
@@ -10692,8 +10692,8 @@
       <c r="L149" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M149">
-        <v>37</v>
+      <c r="M149" t="s">
+        <v>23</v>
       </c>
       <c r="N149" t="s">
         <v>23</v>
@@ -11024,7 +11024,7 @@
         <v>678</v>
       </c>
       <c r="F157" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G157" t="s">
         <v>92</v>
@@ -11044,8 +11044,8 @@
       <c r="L157" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M157">
-        <v>38</v>
+      <c r="M157" t="s">
+        <v>23</v>
       </c>
       <c r="N157" t="s">
         <v>23</v>
@@ -11244,7 +11244,7 @@
         <v>696</v>
       </c>
       <c r="F162" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G162" t="s">
         <v>92</v>
@@ -11264,8 +11264,8 @@
       <c r="L162" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M162">
-        <v>39</v>
+      <c r="M162" t="s">
+        <v>23</v>
       </c>
       <c r="N162" t="s">
         <v>23</v>
@@ -11684,7 +11684,7 @@
         <v>736</v>
       </c>
       <c r="F172" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G172" t="s">
         <v>92</v>
@@ -11704,8 +11704,8 @@
       <c r="L172" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M172">
-        <v>40</v>
+      <c r="M172" t="s">
+        <v>23</v>
       </c>
       <c r="N172" t="s">
         <v>23</v>
@@ -11772,7 +11772,7 @@
         <v>744</v>
       </c>
       <c r="F174" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G174" t="s">
         <v>92</v>
@@ -11792,8 +11792,8 @@
       <c r="L174" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M174">
-        <v>41</v>
+      <c r="M174" t="s">
+        <v>23</v>
       </c>
       <c r="N174" t="s">
         <v>23</v>
@@ -12256,7 +12256,7 @@
         <v>790</v>
       </c>
       <c r="F185" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G185" t="s">
         <v>92</v>
@@ -12276,8 +12276,8 @@
       <c r="L185" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M185">
-        <v>42</v>
+      <c r="M185" t="s">
+        <v>23</v>
       </c>
       <c r="N185" t="s">
         <v>23</v>
@@ -12388,7 +12388,7 @@
         <v>801</v>
       </c>
       <c r="F188" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G188" t="s">
         <v>92</v>
@@ -12408,8 +12408,8 @@
       <c r="L188" s="3" t="s">
         <v>802</v>
       </c>
-      <c r="M188">
-        <v>43</v>
+      <c r="M188" t="s">
+        <v>23</v>
       </c>
       <c r="N188" t="s">
         <v>23</v>
@@ -12564,7 +12564,7 @@
         <v>817</v>
       </c>
       <c r="F192" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G192" t="s">
         <v>92</v>
@@ -12584,8 +12584,8 @@
       <c r="L192" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M192">
-        <v>44</v>
+      <c r="M192" t="s">
+        <v>23</v>
       </c>
       <c r="N192" t="s">
         <v>23</v>
@@ -12740,7 +12740,7 @@
         <v>832</v>
       </c>
       <c r="F196" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G196" t="s">
         <v>92</v>
@@ -12760,8 +12760,8 @@
       <c r="L196" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M196">
-        <v>45</v>
+      <c r="M196" t="s">
+        <v>23</v>
       </c>
       <c r="N196" t="s">
         <v>23</v>
@@ -12784,7 +12784,7 @@
         <v>836</v>
       </c>
       <c r="F197" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G197" t="s">
         <v>92</v>
@@ -12804,8 +12804,8 @@
       <c r="L197" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M197">
-        <v>46</v>
+      <c r="M197" t="s">
+        <v>23</v>
       </c>
       <c r="N197" t="s">
         <v>23</v>
@@ -12828,7 +12828,7 @@
         <v>840</v>
       </c>
       <c r="F198" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G198" t="s">
         <v>92</v>
@@ -12848,8 +12848,8 @@
       <c r="L198" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M198">
-        <v>47</v>
+      <c r="M198" t="s">
+        <v>23</v>
       </c>
       <c r="N198" t="s">
         <v>23</v>
@@ -12916,7 +12916,7 @@
         <v>848</v>
       </c>
       <c r="F200" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G200" t="s">
         <v>92</v>
@@ -12936,8 +12936,8 @@
       <c r="L200" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M200">
-        <v>48</v>
+      <c r="M200" t="s">
+        <v>23</v>
       </c>
       <c r="N200" t="s">
         <v>23</v>
@@ -13048,7 +13048,7 @@
         <v>862</v>
       </c>
       <c r="F203" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G203" t="s">
         <v>92</v>
@@ -13068,8 +13068,8 @@
       <c r="L203" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M203">
-        <v>49</v>
+      <c r="M203" t="s">
+        <v>23</v>
       </c>
       <c r="N203" t="s">
         <v>23</v>
@@ -13136,7 +13136,7 @@
         <v>869</v>
       </c>
       <c r="F205" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G205" t="s">
         <v>92</v>
@@ -13156,8 +13156,8 @@
       <c r="L205" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M205">
-        <v>50</v>
+      <c r="M205" t="s">
+        <v>23</v>
       </c>
       <c r="N205" t="s">
         <v>23</v>
@@ -13224,7 +13224,7 @@
         <v>876</v>
       </c>
       <c r="F207" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G207" t="s">
         <v>92</v>
@@ -13244,8 +13244,8 @@
       <c r="L207" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M207">
-        <v>51</v>
+      <c r="M207" t="s">
+        <v>23</v>
       </c>
       <c r="N207" t="s">
         <v>23</v>
@@ -13532,7 +13532,7 @@
         <v>903</v>
       </c>
       <c r="F214" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G214" t="s">
         <v>92</v>
@@ -13552,8 +13552,8 @@
       <c r="L214" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M214">
-        <v>52</v>
+      <c r="M214" t="s">
+        <v>23</v>
       </c>
       <c r="N214" t="s">
         <v>23</v>
@@ -13664,7 +13664,7 @@
         <v>915</v>
       </c>
       <c r="F217" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G217" t="s">
         <v>92</v>
@@ -13684,8 +13684,8 @@
       <c r="L217" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M217">
-        <v>53</v>
+      <c r="M217" t="s">
+        <v>23</v>
       </c>
       <c r="N217" t="s">
         <v>23</v>
@@ -14324,7 +14324,7 @@
         <v>970</v>
       </c>
       <c r="F232" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G232" t="s">
         <v>92</v>
@@ -14344,8 +14344,8 @@
       <c r="L232" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M232">
-        <v>54</v>
+      <c r="M232" t="s">
+        <v>23</v>
       </c>
       <c r="N232" t="s">
         <v>23</v>
@@ -14412,7 +14412,7 @@
         <v>978</v>
       </c>
       <c r="F234" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G234" t="s">
         <v>92</v>
@@ -14432,8 +14432,8 @@
       <c r="L234" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M234">
-        <v>1</v>
+      <c r="M234" t="s">
+        <v>23</v>
       </c>
       <c r="N234" t="s">
         <v>23</v>
@@ -14632,7 +14632,7 @@
         <v>997</v>
       </c>
       <c r="F239" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G239" t="s">
         <v>92</v>
@@ -14652,8 +14652,8 @@
       <c r="L239" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M239">
-        <v>2</v>
+      <c r="M239" t="s">
+        <v>23</v>
       </c>
       <c r="N239" t="s">
         <v>23</v>
@@ -14676,7 +14676,7 @@
         <v>1000</v>
       </c>
       <c r="F240" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G240" t="s">
         <v>92</v>
@@ -14696,8 +14696,8 @@
       <c r="L240" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M240">
-        <v>3</v>
+      <c r="M240" t="s">
+        <v>23</v>
       </c>
       <c r="N240" t="s">
         <v>23</v>
@@ -14720,7 +14720,7 @@
         <v>1003</v>
       </c>
       <c r="F241" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G241" t="s">
         <v>92</v>
@@ -14740,8 +14740,8 @@
       <c r="L241" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M241">
-        <v>4</v>
+      <c r="M241" t="s">
+        <v>23</v>
       </c>
       <c r="N241" t="s">
         <v>23</v>
@@ -14852,7 +14852,7 @@
         <v>1014</v>
       </c>
       <c r="F244" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G244" t="s">
         <v>92</v>
@@ -14872,8 +14872,8 @@
       <c r="L244" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M244">
-        <v>55</v>
+      <c r="M244" t="s">
+        <v>23</v>
       </c>
       <c r="N244" t="s">
         <v>23</v>
@@ -14984,7 +14984,7 @@
         <v>1028</v>
       </c>
       <c r="F247" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G247" t="s">
         <v>92</v>
@@ -15004,8 +15004,8 @@
       <c r="L247" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M247">
-        <v>5</v>
+      <c r="M247" t="s">
+        <v>23</v>
       </c>
       <c r="N247" t="s">
         <v>23</v>
@@ -15028,7 +15028,7 @@
         <v>1032</v>
       </c>
       <c r="F248" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G248" t="s">
         <v>92</v>
@@ -15048,8 +15048,8 @@
       <c r="L248" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M248">
-        <v>6</v>
+      <c r="M248" t="s">
+        <v>23</v>
       </c>
       <c r="N248" t="s">
         <v>23</v>
@@ -15160,7 +15160,7 @@
         <v>1045</v>
       </c>
       <c r="F251" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G251" t="s">
         <v>92</v>
@@ -15180,8 +15180,8 @@
       <c r="L251" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M251">
-        <v>7</v>
+      <c r="M251" t="s">
+        <v>23</v>
       </c>
       <c r="N251" t="s">
         <v>23</v>
@@ -15248,7 +15248,7 @@
         <v>1052</v>
       </c>
       <c r="F253" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G253" t="s">
         <v>92</v>
@@ -15268,8 +15268,8 @@
       <c r="L253" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M253">
-        <v>56</v>
+      <c r="M253" t="s">
+        <v>23</v>
       </c>
       <c r="N253" t="s">
         <v>23</v>
@@ -15292,7 +15292,7 @@
         <v>1055</v>
       </c>
       <c r="F254" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G254" t="s">
         <v>92</v>
@@ -15312,8 +15312,8 @@
       <c r="L254" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M254">
-        <v>8</v>
+      <c r="M254" t="s">
+        <v>23</v>
       </c>
       <c r="N254" t="s">
         <v>23</v>
@@ -15380,7 +15380,7 @@
         <v>1064</v>
       </c>
       <c r="F256" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G256" t="s">
         <v>92</v>
@@ -15400,8 +15400,8 @@
       <c r="L256" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M256">
-        <v>57</v>
+      <c r="M256" t="s">
+        <v>23</v>
       </c>
       <c r="N256" t="s">
         <v>23</v>
@@ -15424,7 +15424,7 @@
         <v>1067</v>
       </c>
       <c r="F257" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G257" t="s">
         <v>92</v>
@@ -15444,8 +15444,8 @@
       <c r="L257" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M257">
-        <v>9</v>
+      <c r="M257" t="s">
+        <v>23</v>
       </c>
       <c r="N257" t="s">
         <v>23</v>
@@ -15468,7 +15468,7 @@
         <v>1071</v>
       </c>
       <c r="F258" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G258" t="s">
         <v>92</v>
@@ -15488,8 +15488,8 @@
       <c r="L258" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M258">
-        <v>10</v>
+      <c r="M258" t="s">
+        <v>23</v>
       </c>
       <c r="N258" t="s">
         <v>23</v>
@@ -15512,7 +15512,7 @@
         <v>1075</v>
       </c>
       <c r="F259" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G259" t="s">
         <v>92</v>
@@ -15532,8 +15532,8 @@
       <c r="L259" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M259">
-        <v>11</v>
+      <c r="M259" t="s">
+        <v>23</v>
       </c>
       <c r="N259" t="s">
         <v>23</v>
@@ -15556,7 +15556,7 @@
         <v>1079</v>
       </c>
       <c r="F260" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G260" t="s">
         <v>92</v>
@@ -15576,8 +15576,8 @@
       <c r="L260" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M260">
-        <v>58</v>
+      <c r="M260" t="s">
+        <v>23</v>
       </c>
       <c r="N260" t="s">
         <v>23</v>
@@ -15600,7 +15600,7 @@
         <v>1082</v>
       </c>
       <c r="F261" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G261" t="s">
         <v>92</v>
@@ -15620,8 +15620,8 @@
       <c r="L261" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M261">
-        <v>12</v>
+      <c r="M261" t="s">
+        <v>23</v>
       </c>
       <c r="N261" t="s">
         <v>23</v>
@@ -15644,7 +15644,7 @@
         <v>1085</v>
       </c>
       <c r="F262" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G262" t="s">
         <v>92</v>
@@ -15664,8 +15664,8 @@
       <c r="L262" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M262">
-        <v>13</v>
+      <c r="M262" t="s">
+        <v>23</v>
       </c>
       <c r="N262" t="s">
         <v>23</v>
@@ -15732,7 +15732,7 @@
         <v>1091</v>
       </c>
       <c r="F264" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G264" t="s">
         <v>92</v>
@@ -15752,8 +15752,8 @@
       <c r="L264" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M264">
-        <v>59</v>
+      <c r="M264" t="s">
+        <v>23</v>
       </c>
       <c r="N264" t="s">
         <v>23</v>
@@ -15776,7 +15776,7 @@
         <v>1094</v>
       </c>
       <c r="F265" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G265" t="s">
         <v>92</v>
@@ -15796,8 +15796,8 @@
       <c r="L265" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M265">
-        <v>60</v>
+      <c r="M265" t="s">
+        <v>23</v>
       </c>
       <c r="N265" t="s">
         <v>23</v>
@@ -15864,7 +15864,7 @@
         <v>1102</v>
       </c>
       <c r="F267" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G267" t="s">
         <v>92</v>
@@ -15884,8 +15884,8 @@
       <c r="L267" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M267">
-        <v>14</v>
+      <c r="M267" t="s">
+        <v>23</v>
       </c>
       <c r="N267" t="s">
         <v>23</v>
@@ -15908,7 +15908,7 @@
         <v>1105</v>
       </c>
       <c r="F268" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G268" t="s">
         <v>92</v>
@@ -15928,8 +15928,8 @@
       <c r="L268" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M268">
-        <v>15</v>
+      <c r="M268" t="s">
+        <v>23</v>
       </c>
       <c r="N268" t="s">
         <v>23</v>
@@ -15996,7 +15996,7 @@
         <v>1113</v>
       </c>
       <c r="F270" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G270" t="s">
         <v>92</v>
@@ -16016,8 +16016,8 @@
       <c r="L270" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M270">
-        <v>16</v>
+      <c r="M270" t="s">
+        <v>23</v>
       </c>
       <c r="N270" t="s">
         <v>23</v>
@@ -16304,7 +16304,7 @@
         <v>1140</v>
       </c>
       <c r="F277" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G277" t="s">
         <v>92</v>
@@ -16324,8 +16324,8 @@
       <c r="L277" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M277">
-        <v>17</v>
+      <c r="M277" t="s">
+        <v>23</v>
       </c>
       <c r="N277" t="s">
         <v>23</v>
@@ -16348,7 +16348,7 @@
         <v>1143</v>
       </c>
       <c r="F278" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G278" t="s">
         <v>92</v>
@@ -16368,8 +16368,8 @@
       <c r="L278" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M278">
-        <v>18</v>
+      <c r="M278" t="s">
+        <v>23</v>
       </c>
       <c r="N278" t="s">
         <v>23</v>
@@ -16392,7 +16392,7 @@
         <v>1146</v>
       </c>
       <c r="F279" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G279" t="s">
         <v>92</v>
@@ -16412,8 +16412,8 @@
       <c r="L279" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M279">
-        <v>61</v>
+      <c r="M279" t="s">
+        <v>23</v>
       </c>
       <c r="N279" t="s">
         <v>23</v>
@@ -16480,7 +16480,7 @@
         <v>1154</v>
       </c>
       <c r="F281" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G281" t="s">
         <v>92</v>
@@ -16500,8 +16500,8 @@
       <c r="L281" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M281">
-        <v>62</v>
+      <c r="M281" t="s">
+        <v>23</v>
       </c>
       <c r="N281" t="s">
         <v>23</v>
@@ -16568,7 +16568,7 @@
         <v>1162</v>
       </c>
       <c r="F283" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G283" t="s">
         <v>92</v>
@@ -16588,8 +16588,8 @@
       <c r="L283" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M283">
-        <v>63</v>
+      <c r="M283" t="s">
+        <v>23</v>
       </c>
       <c r="N283" t="s">
         <v>23</v>
@@ -16656,7 +16656,7 @@
         <v>1169</v>
       </c>
       <c r="F285" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G285" t="s">
         <v>92</v>
@@ -16676,8 +16676,8 @@
       <c r="L285" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M285">
-        <v>19</v>
+      <c r="M285" t="s">
+        <v>23</v>
       </c>
       <c r="N285" t="s">
         <v>23</v>
@@ -16876,7 +16876,7 @@
         <v>1186</v>
       </c>
       <c r="F290" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G290" t="s">
         <v>92</v>
@@ -16896,8 +16896,8 @@
       <c r="L290" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M290">
-        <v>20</v>
+      <c r="M290" t="s">
+        <v>23</v>
       </c>
       <c r="N290" t="s">
         <v>23</v>
@@ -16920,7 +16920,7 @@
         <v>1190</v>
       </c>
       <c r="F291" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G291" t="s">
         <v>92</v>
@@ -16940,8 +16940,8 @@
       <c r="L291" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M291">
-        <v>21</v>
+      <c r="M291" t="s">
+        <v>23</v>
       </c>
       <c r="N291" t="s">
         <v>23</v>
@@ -16964,7 +16964,7 @@
         <v>1193</v>
       </c>
       <c r="F292" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G292" t="s">
         <v>92</v>
@@ -16984,8 +16984,8 @@
       <c r="L292" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M292">
-        <v>22</v>
+      <c r="M292" t="s">
+        <v>23</v>
       </c>
       <c r="N292" t="s">
         <v>23</v>
@@ -17052,7 +17052,7 @@
         <v>1201</v>
       </c>
       <c r="F294" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G294" t="s">
         <v>92</v>
@@ -17072,7 +17072,7 @@
       <c r="L294" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M294">
+      <c r="M294" t="s">
         <v>23</v>
       </c>
       <c r="N294" t="s">
@@ -17096,7 +17096,7 @@
         <v>1204</v>
       </c>
       <c r="F295" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G295" t="s">
         <v>92</v>
@@ -17116,8 +17116,8 @@
       <c r="L295" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M295">
-        <v>24</v>
+      <c r="M295" t="s">
+        <v>23</v>
       </c>
       <c r="N295" t="s">
         <v>23</v>
@@ -17184,7 +17184,7 @@
         <v>1213</v>
       </c>
       <c r="F297" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G297" t="s">
         <v>92</v>
@@ -17204,8 +17204,8 @@
       <c r="L297" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M297">
-        <v>64</v>
+      <c r="M297" t="s">
+        <v>23</v>
       </c>
       <c r="N297" t="s">
         <v>23</v>
@@ -17228,7 +17228,7 @@
         <v>1217</v>
       </c>
       <c r="F298" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G298" t="s">
         <v>92</v>
@@ -17248,8 +17248,8 @@
       <c r="L298" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M298">
-        <v>65</v>
+      <c r="M298" t="s">
+        <v>23</v>
       </c>
       <c r="N298" t="s">
         <v>23</v>
@@ -17272,7 +17272,7 @@
         <v>1221</v>
       </c>
       <c r="F299" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G299" t="s">
         <v>92</v>
@@ -17292,8 +17292,8 @@
       <c r="L299" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M299">
-        <v>25</v>
+      <c r="M299" t="s">
+        <v>23</v>
       </c>
       <c r="N299" t="s">
         <v>23</v>
@@ -17316,7 +17316,7 @@
         <v>1225</v>
       </c>
       <c r="F300" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G300" t="s">
         <v>92</v>
@@ -17336,8 +17336,8 @@
       <c r="L300" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M300">
-        <v>26</v>
+      <c r="M300" t="s">
+        <v>23</v>
       </c>
       <c r="N300" t="s">
         <v>23</v>
@@ -17360,7 +17360,7 @@
         <v>1229</v>
       </c>
       <c r="F301" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G301" t="s">
         <v>92</v>
@@ -17380,8 +17380,8 @@
       <c r="L301" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M301">
-        <v>66</v>
+      <c r="M301" t="s">
+        <v>23</v>
       </c>
       <c r="N301" t="s">
         <v>23</v>
@@ -17415,7 +17415,7 @@
         <v>1231</v>
       </c>
       <c r="B2">
-        <v>200</v>
+        <v>266</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -17479,7 +17479,7 @@
         <v>1236</v>
       </c>
       <c r="B13">
-        <v>66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>